<commit_message>
feat(auth): add persistent 1-hour local session and logout button
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/tables/Accel_mode_uat.xlsx
+++ b/projects/auto_page/autopageMKII/tables/Accel_mode_uat.xlsx
@@ -15,9 +15,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$D$90</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Processed_Logs'!$A$1:$I$76</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Failed_Orders'!$A$1:$D$776</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Completed_Orders'!$A$1:$C$188</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Processed_Logs'!$A$1:$I$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Failed_Orders'!$A$1:$D$785</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Completed_Orders'!$A$1:$C$190</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sheet4'!$A$1:$A$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -505,7 +505,11 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr"/>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>261004PYNMBJ77</t>
+        </is>
+      </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
           <t>MMV98ST00162100F463S00</t>
@@ -519,7 +523,11 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr"/>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>261004Q63DF97T</t>
+        </is>
+      </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
           <t>MMV98ST001621011B63S00</t>
@@ -529,7 +537,11 @@
       <c r="D7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr"/>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>261004Q9QH1P3V</t>
+        </is>
+      </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
           <t>MMV98ST001611000C73S00</t>
@@ -539,85 +551,141 @@
       <c r="D8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr"/>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>261004QA477QPM</t>
+        </is>
+      </c>
       <c r="B9" s="4" t="inlineStr"/>
       <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr"/>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>261004QDHEFM8R</t>
+        </is>
+      </c>
       <c r="B10" s="4" t="inlineStr"/>
       <c r="C10" s="4" t="inlineStr"/>
       <c r="D10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr"/>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>261004QGFRUB89</t>
+        </is>
+      </c>
       <c r="B11" s="4" t="inlineStr"/>
       <c r="C11" s="4" t="inlineStr"/>
       <c r="D11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr"/>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>261004QKKKN7CP</t>
+        </is>
+      </c>
       <c r="B12" s="4" t="inlineStr"/>
       <c r="C12" s="4" t="inlineStr"/>
       <c r="D12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr"/>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>261004QT6B3W6T</t>
+        </is>
+      </c>
       <c r="B13" s="4" t="inlineStr"/>
       <c r="C13" s="4" t="inlineStr"/>
       <c r="D13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr"/>
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>261004QTYKSRBC</t>
+        </is>
+      </c>
       <c r="B14" s="4" t="inlineStr"/>
       <c r="C14" s="4" t="inlineStr"/>
       <c r="D14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr"/>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>261004QX1BTQAW</t>
+        </is>
+      </c>
       <c r="B15" s="4" t="inlineStr"/>
       <c r="C15" s="4" t="inlineStr"/>
       <c r="D15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr"/>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>261004R2R0Q9HS</t>
+        </is>
+      </c>
       <c r="B16" s="4" t="inlineStr"/>
       <c r="C16" s="4" t="inlineStr"/>
       <c r="D16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr"/>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>261004R3TD9APG</t>
+        </is>
+      </c>
       <c r="B17" s="4" t="inlineStr"/>
       <c r="C17" s="4" t="inlineStr"/>
       <c r="D17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr"/>
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>261005R7HD9X0E</t>
+        </is>
+      </c>
       <c r="B18" s="4" t="inlineStr"/>
       <c r="C18" s="4" t="inlineStr"/>
       <c r="D18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr"/>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>261005R8GY74FG</t>
+        </is>
+      </c>
       <c r="B19" s="4" t="inlineStr"/>
       <c r="C19" s="4" t="inlineStr"/>
       <c r="D19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr"/>
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>261005RFNTFJ0M</t>
+        </is>
+      </c>
       <c r="B20" s="4" t="inlineStr"/>
       <c r="C20" s="4" t="inlineStr"/>
       <c r="D20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr"/>
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>261005RYAJ324R</t>
+        </is>
+      </c>
       <c r="B21" s="4" t="inlineStr"/>
       <c r="C21" s="4" t="inlineStr"/>
       <c r="D21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr"/>
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>261005S1000PVF</t>
+        </is>
+      </c>
       <c r="B22" s="4" t="inlineStr"/>
       <c r="C22" s="4" t="inlineStr"/>
       <c r="D22" s="4" t="inlineStr"/>
@@ -629,31 +697,51 @@
       <c r="D23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr"/>
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>261005S279WG28</t>
+        </is>
+      </c>
       <c r="B24" s="4" t="inlineStr"/>
       <c r="C24" s="4" t="inlineStr"/>
       <c r="D24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr"/>
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>261005S3M1DU26</t>
+        </is>
+      </c>
       <c r="B25" s="4" t="inlineStr"/>
       <c r="C25" s="4" t="inlineStr"/>
       <c r="D25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr"/>
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>261005S561P3G2</t>
+        </is>
+      </c>
       <c r="B26" s="4" t="inlineStr"/>
       <c r="C26" s="4" t="inlineStr"/>
       <c r="D26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr"/>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>261005S6S2BQR4</t>
+        </is>
+      </c>
       <c r="B27" s="4" t="inlineStr"/>
       <c r="C27" s="4" t="inlineStr"/>
       <c r="D27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr"/>
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>261005S7BW2KXG</t>
+        </is>
+      </c>
       <c r="B28" s="4" t="inlineStr"/>
       <c r="C28" s="4" t="inlineStr"/>
       <c r="D28" s="4" t="inlineStr"/>
@@ -1090,7 +1178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I76"/>
+  <dimension ref="A1:I86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="5" min="1" max="1"/>
@@ -1100,7 +1188,7 @@
     <col width="15" customWidth="1" style="5" min="5" max="5"/>
     <col width="20" customWidth="1" style="5" min="6" max="6"/>
     <col width="51" customWidth="1" style="5" min="7" max="7"/>
-    <col width="18" customWidth="1" style="5" min="8" max="8"/>
+    <col width="19" customWidth="1" style="5" min="8" max="8"/>
     <col width="70" customWidth="1" style="5" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -3568,83 +3656,83 @@
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02 17:57:19</t>
+          <t>2026-10-02 17:57:24</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>TH2649086552223</t>
+          <t>TH261896442233P</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>261002HHRWC6MC</t>
-        </is>
-      </c>
-      <c r="D69" s="4" t="inlineStr">
-        <is>
-          <t>TEST_MODE</t>
-        </is>
-      </c>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t>1056.0</t>
-        </is>
-      </c>
+          <t>261002HJMQ3P5U</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr"/>
+      <c r="E69" s="4" t="inlineStr"/>
       <c r="F69" s="4" t="inlineStr"/>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>TEST_SUCCESS (ปรับราคาและใส่คูปองสำเร็จ/All OK)</t>
+          <t>ข้าม (สถานะ: ส่งสินค้าแล้ว)</t>
         </is>
       </c>
       <c r="H69" s="4" t="inlineStr"/>
-      <c r="I69" s="4" t="inlineStr">
-        <is>
-          <t>SP2-001753+SP2-001755: POS=1,056.00/เป้า=1,056.00 [ตรง ✅] | Total: POS=1,056.00/เป้า=1,056.00 [ตรง ✅]</t>
-        </is>
-      </c>
+      <c r="I69" s="4" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02 17:57:24</t>
+          <t>2026-10-02 17:58:22</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>TH261896442233P</t>
+          <t>TH263149080303J</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>261002HJMQ3P5U</t>
-        </is>
-      </c>
-      <c r="D70" s="4" t="inlineStr"/>
-      <c r="E70" s="4" t="inlineStr"/>
+          <t>261002HM5CG6JM</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>TEST_MODE</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>974.0</t>
+        </is>
+      </c>
       <c r="F70" s="4" t="inlineStr"/>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>ข้าม (สถานะ: ส่งสินค้าแล้ว)</t>
+          <t>TEST_SUCCESS (ปรับราคาและใส่คูปองสำเร็จ/All OK)</t>
         </is>
       </c>
       <c r="H70" s="4" t="inlineStr"/>
-      <c r="I70" s="4" t="inlineStr"/>
+      <c r="I70" s="4" t="inlineStr">
+        <is>
+          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598: POS=974.00/เป้า=974.00 [ตรง ✅] | Total: POS=974.00/เป้า=974.00 [ตรง ✅]</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02 17:58:22</t>
+          <t>2026-10-02 17:59:01</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>TH263149080303J</t>
+          <t>TH268776951069O</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>261002HM5CG6JM</t>
+          <t>261002HMFAY2EQ</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -3654,7 +3742,7 @@
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>974.0</t>
+          <t>1056.0</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr"/>
@@ -3666,183 +3754,518 @@
       <c r="H71" s="4" t="inlineStr"/>
       <c r="I71" s="4" t="inlineStr">
         <is>
-          <t>SP2-001703+SP2-001596+SP2-001597+SP2-001598: POS=974.00/เป้า=974.00 [ตรง ✅] | Total: POS=974.00/เป้า=974.00 [ตรง ✅]</t>
+          <t>SP2-001753+SP2-001755: POS=1,056.00/เป้า=1,056.00 [ตรง ✅] | Total: POS=1,056.00/เป้า=1,056.00 [ตรง ✅]</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02 17:59:01</t>
+          <t>2026-10-02 17:59:08</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>TH268776951069O</t>
+          <t>TH260983554839J</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>261002HMFAY2EQ</t>
-        </is>
-      </c>
-      <c r="D72" s="4" t="inlineStr">
-        <is>
-          <t>TEST_MODE</t>
-        </is>
-      </c>
-      <c r="E72" s="4" t="inlineStr">
-        <is>
-          <t>1056.0</t>
-        </is>
-      </c>
+          <t>261002HN2N0SB4</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr"/>
+      <c r="E72" s="4" t="inlineStr"/>
       <c r="F72" s="4" t="inlineStr"/>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>TEST_SUCCESS (ปรับราคาและใส่คูปองสำเร็จ/All OK)</t>
+          <t>ข้าม (สถานะ: ส่งสินค้าแล้ว)</t>
         </is>
       </c>
       <c r="H72" s="4" t="inlineStr"/>
-      <c r="I72" s="4" t="inlineStr">
-        <is>
-          <t>SP2-001753+SP2-001755: POS=1,056.00/เป้า=1,056.00 [ตรง ✅] | Total: POS=1,056.00/เป้า=1,056.00 [ตรง ✅]</t>
-        </is>
-      </c>
+      <c r="I72" s="4" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02 17:59:08</t>
+          <t>2026-10-02 17:59:39</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>TH260983554839J</t>
+          <t>TH2613592229088</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>261002HN2N0SB4</t>
-        </is>
-      </c>
-      <c r="D73" s="4" t="inlineStr"/>
-      <c r="E73" s="4" t="inlineStr"/>
+          <t>261002HNMRU6N2</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>TEST_MODE</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>278.0</t>
+        </is>
+      </c>
       <c r="F73" s="4" t="inlineStr"/>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>ข้าม (สถานะ: ส่งสินค้าแล้ว)</t>
+          <t>TEST_SUCCESS (ปรับราคาและใส่คูปองสำเร็จ/All OK)</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr"/>
-      <c r="I73" s="4" t="inlineStr"/>
+      <c r="I73" s="4" t="inlineStr">
+        <is>
+          <t>SP4-000302: POS=139.00/เป้า=139.00 [ตรง ✅] | Total: POS=278.00/เป้า=278.00 [ตรง ✅]</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02 17:59:39</t>
+          <t>2026-10-02 17:59:45</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>TH2613592229088</t>
+          <t>TH040697FCG04D</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>261002HNMRU6N2</t>
-        </is>
-      </c>
-      <c r="D74" s="4" t="inlineStr">
-        <is>
-          <t>TEST_MODE</t>
-        </is>
-      </c>
-      <c r="E74" s="4" t="inlineStr">
-        <is>
-          <t>278.0</t>
-        </is>
-      </c>
+          <t>261002HPM17BKR</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr"/>
+      <c r="E74" s="4" t="inlineStr"/>
       <c r="F74" s="4" t="inlineStr"/>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>TEST_SUCCESS (ปรับราคาและใส่คูปองสำเร็จ/All OK)</t>
+          <t>ข้าม (สถานะ: ส่งสินค้าแล้ว)</t>
         </is>
       </c>
       <c r="H74" s="4" t="inlineStr"/>
-      <c r="I74" s="4" t="inlineStr">
-        <is>
-          <t>SP4-000302: POS=139.00/เป้า=139.00 [ตรง ✅] | Total: POS=278.00/เป้า=278.00 [ตรง ✅]</t>
-        </is>
-      </c>
+      <c r="I74" s="4" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02 17:59:45</t>
+          <t>2026-10-02 18:00:26</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>TH040697FCG04D</t>
+          <t>TH261278054656S</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>261002HPM17BKR</t>
-        </is>
-      </c>
-      <c r="D75" s="4" t="inlineStr"/>
-      <c r="E75" s="4" t="inlineStr"/>
+          <t>261002HSH1MCYP</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>TEST_MODE</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>1603.0</t>
+        </is>
+      </c>
       <c r="F75" s="4" t="inlineStr"/>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>ข้าม (สถานะ: ส่งสินค้าแล้ว)</t>
+          <t>TEST_SUCCESS (ปรับราคาและใส่คูปองสำเร็จ/All OK)</t>
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr"/>
-      <c r="I75" s="4" t="inlineStr"/>
+      <c r="I75" s="4" t="inlineStr">
+        <is>
+          <t>SP1-001113: POS=1,603.00/เป้า=1,603.00 [ตรง ✅] | Total: POS=1,603.00/เป้า=1,603.00 [ตรง ✅]</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02 18:00:26</t>
-        </is>
-      </c>
-      <c r="B76" s="4" t="inlineStr">
-        <is>
-          <t>TH261278054656S</t>
-        </is>
-      </c>
+          <t>2026-10-05 10:35:06</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr"/>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>261002HSH1MCYP</t>
-        </is>
-      </c>
-      <c r="D76" s="4" t="inlineStr">
-        <is>
-          <t>TEST_MODE</t>
-        </is>
-      </c>
-      <c r="E76" s="4" t="inlineStr">
-        <is>
-          <t>1603.0</t>
-        </is>
-      </c>
+          <t>261002HSQNAN0G</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr"/>
+      <c r="E76" s="4" t="inlineStr"/>
       <c r="F76" s="4" t="inlineStr"/>
       <c r="G76" s="4" t="inlineStr">
         <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="H76" s="4" t="inlineStr">
+        <is>
+          <t>ORDER_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="I76" s="4" t="inlineStr">
+        <is>
+          <t>Error in order_search (ValueError): ไม่พบออเดอร์ 261002HSQNAN0G ในไฟล์นำเข้า (Export File)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:35:08</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr"/>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>261002HST6DBDD</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr"/>
+      <c r="E77" s="4" t="inlineStr"/>
+      <c r="F77" s="4" t="inlineStr"/>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>ORDER_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="I77" s="4" t="inlineStr">
+        <is>
+          <t>Error in order_search (ValueError): ไม่พบออเดอร์ 261002HST6DBDD ในไฟล์นำเข้า (Export File)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:35:09</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr"/>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>261002HTPHAVFD</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr"/>
+      <c r="E78" s="4" t="inlineStr"/>
+      <c r="F78" s="4" t="inlineStr"/>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="H78" s="4" t="inlineStr">
+        <is>
+          <t>ORDER_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="I78" s="4" t="inlineStr">
+        <is>
+          <t>Error in order_search (ValueError): ไม่พบออเดอร์ 261002HTPHAVFD ในไฟล์นำเข้า (Export File)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:35:11</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr"/>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>261002HXGQF53W</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr"/>
+      <c r="E79" s="4" t="inlineStr"/>
+      <c r="F79" s="4" t="inlineStr"/>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>ORDER_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="I79" s="4" t="inlineStr">
+        <is>
+          <t>Error in order_search (ValueError): ไม่พบออเดอร์ 261002HXGQF53W ในไฟล์นำเข้า (Export File)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:35:12</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr"/>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>261002HYAXPRKH</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr"/>
+      <c r="E80" s="4" t="inlineStr"/>
+      <c r="F80" s="4" t="inlineStr"/>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="H80" s="4" t="inlineStr">
+        <is>
+          <t>ORDER_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="I80" s="4" t="inlineStr">
+        <is>
+          <t>Error in order_search (ValueError): ไม่พบออเดอร์ 261002HYAXPRKH ในไฟล์นำเข้า (Export File)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:35:13</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr"/>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>261002J054W3CE</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr"/>
+      <c r="E81" s="4" t="inlineStr"/>
+      <c r="F81" s="4" t="inlineStr"/>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>ORDER_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="I81" s="4" t="inlineStr">
+        <is>
+          <t>Error in order_search (ValueError): ไม่พบออเดอร์ 261002J054W3CE ในไฟล์นำเข้า (Export File)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:35:15</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr"/>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>261002J07DEMAS</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr"/>
+      <c r="E82" s="4" t="inlineStr"/>
+      <c r="F82" s="4" t="inlineStr"/>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="H82" s="4" t="inlineStr">
+        <is>
+          <t>ORDER_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="I82" s="4" t="inlineStr">
+        <is>
+          <t>Error in order_search (ValueError): ไม่พบออเดอร์ 261002J07DEMAS ในไฟล์นำเข้า (Export File)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:36:51</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>TH2649086552223</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>261002HHRWC6MC</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>TEST_MODE</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>1056.0</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr"/>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
           <t>TEST_SUCCESS (ปรับราคาและใส่คูปองสำเร็จ/All OK)</t>
         </is>
       </c>
-      <c r="H76" s="4" t="inlineStr"/>
-      <c r="I76" s="4" t="inlineStr">
-        <is>
-          <t>SP1-001113: POS=1,603.00/เป้า=1,603.00 [ตรง ✅] | Total: POS=1,603.00/เป้า=1,603.00 [ตรง ✅]</t>
+      <c r="H83" s="4" t="inlineStr"/>
+      <c r="I83" s="4" t="inlineStr">
+        <is>
+          <t>SP2-001753+SP2-001755: POS=1,056.00/เป้า=1,056.00 [ตรง ✅] | Total: POS=1,056.00/เป้า=1,056.00 [ตรง ✅]</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:37:27</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>TH266344451938Z</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>261002JEPP9507</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>TEST_MODE</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>1056.0</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr"/>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>TEST_SUCCESS (ปรับราคาและใส่คูปองสำเร็จ/All OK)</t>
+        </is>
+      </c>
+      <c r="H84" s="4" t="inlineStr"/>
+      <c r="I84" s="4" t="inlineStr">
+        <is>
+          <t>SP2-001753+SP2-001755: POS=1,056.00/เป้า=1,056.00 [ตรง ✅] | Total: POS=1,056.00/เป้า=1,056.00 [ตรง ✅]</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:38:02</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>TH269692353735Y</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>261003K6J8B8H5</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr"/>
+      <c r="E85" s="4" t="inlineStr"/>
+      <c r="F85" s="4" t="inlineStr"/>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>PRICE_MISMATCH</t>
+        </is>
+      </c>
+      <c r="I85" s="4" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not set for SKU: SP2-001753+SP2-001755 (วันที่: 2026-10-03 00:04, ราคาที่ต้องออกบิล: 993.0)
+SHOPEE เวลาสั่งซื้อ 2026-10-03 00:04
+SP2-001753+SP2-001755 CANON ตลับหมึกรุ่น  PG-47 BK / CANON Ink CL-57 CO และ PACK คู่ 2 สี
+ยิงขายขึ้น 1,240.00 บาท
+ลูกค้าซื้อราคา 993.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:38:51</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>TH260526331025L</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>261003ND0STEU0</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>TEST_MODE</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="inlineStr">
+        <is>
+          <t>1280.0</t>
+        </is>
+      </c>
+      <c r="F86" s="4" t="inlineStr"/>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>TEST_SUCCESS (ปรับราคาและใส่คูปองสำเร็จ/All OK)</t>
+        </is>
+      </c>
+      <c r="H86" s="4" t="inlineStr"/>
+      <c r="I86" s="4" t="inlineStr">
+        <is>
+          <t>SP2-001610+SP2-001611+SP2-001612+SP2-001613: POS=1,280.00/เป้า=1,280.00 [ตรง ✅] | Total: POS=1,280.00/เป้า=1,280.00 [ตรง ✅]</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I76"/>
+  <autoFilter ref="A1:I86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3853,7 +4276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D776"/>
+  <dimension ref="A1:D785"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="5" min="1" max="1"/>
@@ -24509,8 +24932,216 @@
         </is>
       </c>
     </row>
+    <row r="777">
+      <c r="A777" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:35:07</t>
+        </is>
+      </c>
+      <c r="B777" s="4" t="inlineStr">
+        <is>
+          <t>ORDER_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="C777" s="4" t="inlineStr">
+        <is>
+          <t>261002HSQNAN0G</t>
+        </is>
+      </c>
+      <c r="D777" s="4" t="inlineStr">
+        <is>
+          <t>Error in order_search (ValueError): ไม่พบออเดอร์ 261002HSQNAN0G ในไฟล์นำเข้า (Export File)</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:35:08</t>
+        </is>
+      </c>
+      <c r="B778" s="4" t="inlineStr">
+        <is>
+          <t>ORDER_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="C778" s="4" t="inlineStr">
+        <is>
+          <t>261002HST6DBDD</t>
+        </is>
+      </c>
+      <c r="D778" s="4" t="inlineStr">
+        <is>
+          <t>Error in order_search (ValueError): ไม่พบออเดอร์ 261002HST6DBDD ในไฟล์นำเข้า (Export File)</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:35:10</t>
+        </is>
+      </c>
+      <c r="B779" s="4" t="inlineStr">
+        <is>
+          <t>ORDER_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="C779" s="4" t="inlineStr">
+        <is>
+          <t>261002HTPHAVFD</t>
+        </is>
+      </c>
+      <c r="D779" s="4" t="inlineStr">
+        <is>
+          <t>Error in order_search (ValueError): ไม่พบออเดอร์ 261002HTPHAVFD ในไฟล์นำเข้า (Export File)</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:35:11</t>
+        </is>
+      </c>
+      <c r="B780" s="4" t="inlineStr">
+        <is>
+          <t>ORDER_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="C780" s="4" t="inlineStr">
+        <is>
+          <t>261002HXGQF53W</t>
+        </is>
+      </c>
+      <c r="D780" s="4" t="inlineStr">
+        <is>
+          <t>Error in order_search (ValueError): ไม่พบออเดอร์ 261002HXGQF53W ในไฟล์นำเข้า (Export File)</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:35:13</t>
+        </is>
+      </c>
+      <c r="B781" s="4" t="inlineStr">
+        <is>
+          <t>ORDER_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="C781" s="4" t="inlineStr">
+        <is>
+          <t>261002HYAXPRKH</t>
+        </is>
+      </c>
+      <c r="D781" s="4" t="inlineStr">
+        <is>
+          <t>Error in order_search (ValueError): ไม่พบออเดอร์ 261002HYAXPRKH ในไฟล์นำเข้า (Export File)</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:35:14</t>
+        </is>
+      </c>
+      <c r="B782" s="4" t="inlineStr">
+        <is>
+          <t>ORDER_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="C782" s="4" t="inlineStr">
+        <is>
+          <t>261002J054W3CE</t>
+        </is>
+      </c>
+      <c r="D782" s="4" t="inlineStr">
+        <is>
+          <t>Error in order_search (ValueError): ไม่พบออเดอร์ 261002J054W3CE ในไฟล์นำเข้า (Export File)</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:35:15</t>
+        </is>
+      </c>
+      <c r="B783" s="4" t="inlineStr">
+        <is>
+          <t>ORDER_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="C783" s="4" t="inlineStr">
+        <is>
+          <t>261002J07DEMAS</t>
+        </is>
+      </c>
+      <c r="D783" s="4" t="inlineStr">
+        <is>
+          <t>Error in order_search (ValueError): ไม่พบออเดอร์ 261002J07DEMAS ในไฟล์นำเข้า (Export File)</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:37:59</t>
+        </is>
+      </c>
+      <c r="B784" s="4" t="inlineStr">
+        <is>
+          <t>PRICE_MISMATCH</t>
+        </is>
+      </c>
+      <c r="C784" s="4" t="inlineStr">
+        <is>
+          <t>261003K6J8B8H5</t>
+        </is>
+      </c>
+      <c r="D784" s="4" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not set for SKU: SP2-001753+SP2-001755 (วันที่: 2026-10-03 00:04, ราคาที่ต้องออกบิล: 993.0)
+SHOPEE เวลาสั่งซื้อ 2026-10-03 00:04
+SP2-001753+SP2-001755 CANON ตลับหมึกรุ่น  PG-47 BK / CANON Ink CL-57 CO และ PACK คู่ 2 สี
+ยิงขายขึ้น 1,240.00 บาท
+ลูกค้าซื้อราคา 993.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:38:02</t>
+        </is>
+      </c>
+      <c r="B785" s="4" t="inlineStr">
+        <is>
+          <t>PRICE_MISMATCH</t>
+        </is>
+      </c>
+      <c r="C785" s="4" t="inlineStr">
+        <is>
+          <t>261003K6J8B8H5</t>
+        </is>
+      </c>
+      <c r="D785" s="4" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not set for SKU: SP2-001753+SP2-001755 (วันที่: 2026-10-03 00:04, ราคาที่ต้องออกบิล: 993.0)
+SHOPEE เวลาสั่งซื้อ 2026-10-03 00:04
+SP2-001753+SP2-001755 CANON ตลับหมึกรุ่น  PG-47 BK / CANON Ink CL-57 CO และ PACK คู่ 2 สี
+ยิงขายขึ้น 1,240.00 บาท
+ลูกค้าซื้อราคา 993.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D776"/>
+  <autoFilter ref="A1:D785"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24521,7 +25152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C188"/>
+  <dimension ref="A1:C190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="5" min="1" max="1"/>
@@ -27592,46 +28223,46 @@
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02 17:57:19</t>
+          <t>2026-10-02 17:57:24</t>
         </is>
       </c>
       <c r="B181" s="4" t="inlineStr">
         <is>
-          <t>261002HHRWC6MC</t>
+          <t>261002HJMQ3P5U</t>
         </is>
       </c>
       <c r="C181" s="4" t="inlineStr">
         <is>
-          <t>TEST_SUCCESS (ปรับราคาและใส่คูปองสำเร็จ/All OK)</t>
+          <t>ข้าม (สถานะ: ส่งสินค้าแล้ว)</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02 17:57:24</t>
+          <t>2026-10-02 17:58:22</t>
         </is>
       </c>
       <c r="B182" s="4" t="inlineStr">
         <is>
-          <t>261002HJMQ3P5U</t>
+          <t>261002HM5CG6JM</t>
         </is>
       </c>
       <c r="C182" s="4" t="inlineStr">
         <is>
-          <t>ข้าม (สถานะ: ส่งสินค้าแล้ว)</t>
+          <t>TEST_SUCCESS (ปรับราคาและใส่คูปองสำเร็จ/All OK)</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02 17:58:22</t>
+          <t>2026-10-02 17:59:01</t>
         </is>
       </c>
       <c r="B183" s="4" t="inlineStr">
         <is>
-          <t>261002HM5CG6JM</t>
+          <t>261002HMFAY2EQ</t>
         </is>
       </c>
       <c r="C183" s="4" t="inlineStr">
@@ -27643,80 +28274,80 @@
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02 17:59:01</t>
+          <t>2026-10-02 17:59:08</t>
         </is>
       </c>
       <c r="B184" s="4" t="inlineStr">
         <is>
-          <t>261002HMFAY2EQ</t>
+          <t>261002HN2N0SB4</t>
         </is>
       </c>
       <c r="C184" s="4" t="inlineStr">
         <is>
-          <t>TEST_SUCCESS (ปรับราคาและใส่คูปองสำเร็จ/All OK)</t>
+          <t>ข้าม (สถานะ: ส่งสินค้าแล้ว)</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02 17:59:08</t>
+          <t>2026-10-02 17:59:39</t>
         </is>
       </c>
       <c r="B185" s="4" t="inlineStr">
         <is>
-          <t>261002HN2N0SB4</t>
+          <t>261002HNMRU6N2</t>
         </is>
       </c>
       <c r="C185" s="4" t="inlineStr">
         <is>
-          <t>ข้าม (สถานะ: ส่งสินค้าแล้ว)</t>
+          <t>TEST_SUCCESS (ปรับราคาและใส่คูปองสำเร็จ/All OK)</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02 17:59:39</t>
+          <t>2026-10-02 17:59:45</t>
         </is>
       </c>
       <c r="B186" s="4" t="inlineStr">
         <is>
-          <t>261002HNMRU6N2</t>
+          <t>261002HPM17BKR</t>
         </is>
       </c>
       <c r="C186" s="4" t="inlineStr">
         <is>
-          <t>TEST_SUCCESS (ปรับราคาและใส่คูปองสำเร็จ/All OK)</t>
+          <t>ข้าม (สถานะ: ส่งสินค้าแล้ว)</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02 17:59:45</t>
+          <t>2026-10-02 18:00:26</t>
         </is>
       </c>
       <c r="B187" s="4" t="inlineStr">
         <is>
-          <t>261002HPM17BKR</t>
+          <t>261002HSH1MCYP</t>
         </is>
       </c>
       <c r="C187" s="4" t="inlineStr">
         <is>
-          <t>ข้าม (สถานะ: ส่งสินค้าแล้ว)</t>
+          <t>TEST_SUCCESS (ปรับราคาและใส่คูปองสำเร็จ/All OK)</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02 18:00:26</t>
+          <t>2026-10-05 10:36:51</t>
         </is>
       </c>
       <c r="B188" s="4" t="inlineStr">
         <is>
-          <t>261002HSH1MCYP</t>
+          <t>261002HHRWC6MC</t>
         </is>
       </c>
       <c r="C188" s="4" t="inlineStr">
@@ -27725,8 +28356,42 @@
         </is>
       </c>
     </row>
+    <row r="189">
+      <c r="A189" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:37:27</t>
+        </is>
+      </c>
+      <c r="B189" s="4" t="inlineStr">
+        <is>
+          <t>261002JEPP9507</t>
+        </is>
+      </c>
+      <c r="C189" s="4" t="inlineStr">
+        <is>
+          <t>TEST_SUCCESS (ปรับราคาและใส่คูปองสำเร็จ/All OK)</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:38:51</t>
+        </is>
+      </c>
+      <c r="B190" s="4" t="inlineStr">
+        <is>
+          <t>261003ND0STEU0</t>
+        </is>
+      </c>
+      <c r="C190" s="4" t="inlineStr">
+        <is>
+          <t>TEST_SUCCESS (ปรับราคาและใส่คูปองสำเร็จ/All OK)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C188"/>
+  <autoFilter ref="A1:C190"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>